<commit_message>
Add original Corona annual report with explicit financial-data limits
</commit_message>
<xml_diff>
--- a/data/mfa-preliminary.xlsx
+++ b/data/mfa-preliminary.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reported collections'!$A$1:$AF$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Source index'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Source index'!$A$1:$N$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Residential cash'!$A$1:$AF$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Capital spending'!$A$1:$R$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Funded shares'!$A$1:$R$1</definedName>
@@ -951,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1230,12 +1230,74 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>corona-2024-25</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>City of Corona</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>annual_developer_fee_report</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>libraries; transportation; drainage; law_enforcement; fire_emergency_facilities; parks_recreation_open_space; community_facilities; water; sewer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>AB1600 Development Impact Fees Annual Report: Year ended June 30, 2025</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://cdn.prod.website-files.com/65799af8ef225180fdf1ba2e/69384a264b4f0fec01050e8b_AB1600%20report%20FY2025.pdf</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>sources/corona-2024-25.pdf</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>df6de2fe78cfdf6c5924f6568589330315f9544d08fad3df2fa7de2d3da879eb</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>2879030</v>
+      </c>
+      <c r="L5" t="n">
+        <v>24</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>source_only_figures_withheld</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:N5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>